<commit_message>
Compact preview, pinyin college order and sourced Kotone decoration
</commit_message>
<xml_diff>
--- a/examples/fictional-students.xlsx
+++ b/examples/fictional-students.xlsx
@@ -224,12 +224,12 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">示例学生甲</t>
+          <t xml:space="preserve">张三</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEMO-0001</t>
+          <t xml:space="preserve">52x0001</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -239,7 +239,7 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">示例导师甲</t>
+          <t xml:space="preserve">陈老师</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -290,17 +290,17 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">信息技术类</t>
+          <t xml:space="preserve">机械控制自动化类</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">示例学生乙</t>
+          <t xml:space="preserve">李四</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEMO-0002</t>
+          <t xml:space="preserve">52x0002</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -310,7 +310,7 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">示例导师乙</t>
+          <t xml:space="preserve">林老师</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -366,12 +366,12 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">示例学生丙</t>
+          <t xml:space="preserve">王五</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEMO-0003</t>
+          <t xml:space="preserve">52x0003</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -381,7 +381,7 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">示例导师丙</t>
+          <t xml:space="preserve">黄老师</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -432,17 +432,17 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">文史哲经管类</t>
+          <t xml:space="preserve">人文社科类</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">示例学生丁</t>
+          <t xml:space="preserve">赵六</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEMO-0004</t>
+          <t xml:space="preserve">52x0004</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -452,7 +452,7 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">示例导师丁</t>
+          <t xml:space="preserve">吴老师</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
@@ -508,12 +508,12 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">示例学生戊</t>
+          <t xml:space="preserve">孙七</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEMO-0005</t>
+          <t xml:space="preserve">52x0005</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
@@ -523,7 +523,7 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">示例导师戊</t>
+          <t xml:space="preserve">郑老师</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
@@ -574,17 +574,17 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">文史哲经管类</t>
+          <t xml:space="preserve">人文社科类</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">示例学生己</t>
+          <t xml:space="preserve">周八</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEMO-0006</t>
+          <t xml:space="preserve">52x0006</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
@@ -594,7 +594,7 @@
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">示例导师己</t>
+          <t xml:space="preserve">何老师</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">

</xml_diff>